<commit_message>
perf: keep the cells of a sheet with a pivot table (#721)
A pivot table no longer excludes its sheet from the fast path of #702. XLibur does not lay a pivot table out: the load reads no pivot values into the cells, and a change to a pivot table is written to its own part, so the cells a save would write do not depend on it.

Two reference outputs change: their pivot sheets now keep the cells as the input had them, with the file's own cellXfs indices (pivotButton kept where the input had it), its rows' heights without an added customHeight, and the styled blank cells the rewrite dropped.
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Other/PivotTableReferenceFiles/TwoPivotTablesWithSingleSource/output.xlsx
+++ b/XLibur.Tests/Resource/Other/PivotTableReferenceFiles/TwoPivotTablesWithSingleSource/output.xlsx
@@ -7115,135 +7115,135 @@
     <x:col min="5" max="5" width="15.5" customWidth="1"/>
     <x:col min="6" max="6" width="13.832031" customWidth="1"/>
   </x:cols>
-  <x:sheetData>
-    <x:row r="3" spans="1:8">
-      <x:c r="B3" s="4"/>
-      <x:c r="C3" s="6"/>
-      <x:c r="D3" s="6"/>
-      <x:c r="E3" s="4" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="F3" s="6" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="G3" s="6"/>
-      <x:c r="H3" s="7"/>
-    </x:row>
-    <x:row r="4" spans="1:8" ht="11.25" customHeight="1">
-      <x:c r="B4" s="9"/>
-      <x:c r="C4" s="8"/>
-      <x:c r="D4" s="8"/>
-      <x:c r="E4" s="11" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F4" s="6"/>
-      <x:c r="G4" s="11" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="H4" s="40" t="s">
-        <x:v>15</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:8" ht="25.5" customHeight="1">
-      <x:c r="B5" s="13" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C5" s="13" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D5" s="13" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E5" s="13" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="F5" s="13" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="G5" s="9"/>
-      <x:c r="H5" s="41"/>
-    </x:row>
-    <x:row r="6" spans="1:8">
-      <x:c r="B6" s="3" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C6" s="3" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D6" s="3" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="E6" s="3">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F6" s="3">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G6" s="3">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H6" s="3">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:8">
-      <x:c r="B7" s="3"/>
-      <x:c r="C7" s="3" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="D7" s="3"/>
-      <x:c r="E7" s="3">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F7" s="3">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G7" s="3">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H7" s="3">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:8" ht="12" customHeight="1">
-      <x:c r="B8" s="3" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C8" s="3"/>
-      <x:c r="D8" s="3"/>
-      <x:c r="E8" s="3">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F8" s="3">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G8" s="3">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H8" s="3">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" spans="1:8" ht="12.75" customHeight="1">
-      <x:c r="B9" s="3" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C9" s="3"/>
-      <x:c r="D9" s="3"/>
-      <x:c r="E9" s="3">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F9" s="3">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G9" s="3">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H9" s="3">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
+  <sheetData xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+    <row r="3" spans="2:8">
+      <c r="B3" s="4"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="10"/>
+      <c r="H3" s="7"/>
+    </row>
+    <row r="4" spans="2:8" ht="11.25" customHeight="1">
+      <c r="B4" s="9"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="37" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="38"/>
+      <c r="G4" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="40" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" ht="25.5">
+      <c r="B5" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="39"/>
+      <c r="H5" s="41"/>
+    </row>
+    <row r="6" spans="2:8">
+      <c r="B6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="3">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3">
+        <v>0</v>
+      </c>
+      <c r="G6" s="3">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8">
+      <c r="B7" s="3"/>
+      <c r="C7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3">
+        <v>0</v>
+      </c>
+      <c r="F7" s="3">
+        <v>0</v>
+      </c>
+      <c r="G7" s="3">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" ht="12">
+      <c r="B8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3">
+        <v>0</v>
+      </c>
+      <c r="F8" s="3">
+        <v>0</v>
+      </c>
+      <c r="G8" s="3">
+        <v>0</v>
+      </c>
+      <c r="H8" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" ht="12.75">
+      <c r="B9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3">
+        <v>0</v>
+      </c>
+      <c r="F9" s="3">
+        <v>0</v>
+      </c>
+      <c r="G9" s="3">
+        <v>0</v>
+      </c>
+      <c r="H9" s="3">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <x:mergeCells count="7">
     <x:mergeCell ref="E4:F4"/>
     <x:mergeCell ref="G4:G5"/>
@@ -7270,70 +7270,77 @@
     <x:col min="4" max="4" width="20.5" customWidth="1"/>
     <x:col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
   </x:cols>
-  <x:sheetData>
-    <x:row r="4" spans="1:5">
-      <x:c r="B4" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C4" s="6"/>
-      <x:c r="D4" s="4" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E4" s="7"/>
-    </x:row>
-    <x:row r="5" spans="1:5">
-      <x:c r="B5" s="4" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C5" s="4" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D5" s="4" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="E5" s="4" t="s">
-        <x:v>11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:5">
-      <x:c r="B6" s="11" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C6" s="11" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="D6" s="11">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E6" s="11">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:5" ht="11.25" customHeight="1">
-      <x:c r="B7" s="11" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C7" s="11"/>
-      <x:c r="D7" s="11">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E7" s="11">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:5">
-      <x:c r="B8" s="11" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C8" s="11"/>
-      <x:c r="D8" s="11">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E8" s="11">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
+  <sheetData xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+    <row r="1" spans="2:5" s="1" customFormat="1"/>
+    <row r="4" spans="2:5">
+      <c r="B4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="10"/>
+      <c r="D4" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="7"/>
+    </row>
+    <row r="5" spans="2:5">
+      <c r="B5" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5">
+      <c r="B6" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="11">
+        <v>0</v>
+      </c>
+      <c r="E6" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" ht="11.25" customHeight="1">
+      <c r="B7" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11">
+        <v>0</v>
+      </c>
+      <c r="E7" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5">
+      <c r="B8" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11">
+        <v>0</v>
+      </c>
+      <c r="E8" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5">
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+    </row>
+  </sheetData>
   <x:mergeCells count="2">
     <x:mergeCell ref="B7:C7"/>
     <x:mergeCell ref="B8:C8"/>

</xml_diff>